<commit_message>
sample sheed fix first row only
</commit_message>
<xml_diff>
--- a/TCID50.xlsx
+++ b/TCID50.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://charitede-my.sharepoint.com/personal/niklas_endres_charite_de/Documents/Experiments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niklas/code/TCID50/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="179" documentId="8_{098CEDCD-0569-5F48-AC56-088500C5A289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84FD5792-398E-2842-AC2A-443C1FE16390}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643A12AE-9353-044F-AA7C-811BF62FFBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="17960" xr2:uid="{36794AAE-150A-424E-812A-4651D4CE985E}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="28800" windowHeight="17960" xr2:uid="{36794AAE-150A-424E-812A-4651D4CE985E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A:$U</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Sheet1!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Sheet1!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -399,7 +399,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4698,7 +4698,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.25" right="0.25" top="0.59722222222222221" bottom="0.3611111111111111" header="0.3" footer="0.3"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.59055118110236227" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos Narrow (Body),Regular"&amp;16Experiment: &amp;C&amp;"Aptos Narrow (Body),Regular"&amp;16Page &amp;P</oddHeader>

</xml_diff>